<commit_message>
Add player jersey numbers
</commit_message>
<xml_diff>
--- a/2026颶風騎士收支明細費用表.xlsx
+++ b/2026颶風騎士收支明細費用表.xlsx
@@ -1,14 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admir\Desktop\Project\Hurricane Knight\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B013C9B-497B-45E6-8BB8-B602718CAD01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="隊費及儲值金收費紀錄" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="比賽逐場費用明細" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="隊費明細" sheetId="3" r:id="rId7"/>
+    <sheet name="隊費及儲值金收費紀錄" sheetId="1" r:id="rId1"/>
+    <sheet name="比賽逐場費用明細" sheetId="2" r:id="rId2"/>
+    <sheet name="隊費明細" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -216,30 +241,41 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF434343"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -247,7 +283,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -287,28 +323,38 @@
     </fill>
   </fills>
   <borders count="9">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF674EA7"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF292F50"/>
       </top>
       <bottom style="thin">
         <color rgb="FF292F50"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FFFFFFFF"/>
       </top>
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -323,17 +369,20 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FFF6F8F9"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FFF6F8F9"/>
       </top>
       <bottom style="thin">
         <color rgb="FFF6F8F9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -348,6 +397,7 @@
       <bottom style="thin">
         <color rgb="FFF6F8F9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -362,17 +412,20 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FFFFFFFF"/>
       </top>
       <bottom style="thin">
         <color rgb="FF292F50"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -387,195 +440,197 @@
       <bottom style="thin">
         <color rgb="FF292F50"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="48">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="4" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="6" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="7" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="7" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="8" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="16">
     <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
+      <border>
+        <left style="thin">
+          <color rgb="FF373F6B"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF373F6B"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF373F6B"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF373F6B"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
-      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF373F6B"/>
           <bgColor rgb="FF373F6B"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <border/>
     </dxf>
     <dxf>
       <border>
@@ -593,46 +648,146 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF373F6B"/>
+          <bgColor rgb="FF373F6B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF373F6B"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF373F6B"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF373F6B"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF373F6B"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF373F6B"/>
+          <bgColor rgb="FF373F6B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF373F6B"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF373F6B"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF373F6B"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF373F6B"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF373F6B"/>
+          <bgColor rgb="FF373F6B"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="4">
-    <tableStyle count="4" pivot="0" name="隊費明細-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="隊費明細-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="12"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="secondRowStripe" dxfId="13"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="隊費及儲值金收費紀錄-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="隊費及儲值金收費紀錄-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="11"/>
+      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="secondRowStripe" dxfId="9"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="比賽逐場費用明細-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="比賽逐場費用明細-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+      <tableStyleElement type="firstRowStripe" dxfId="6"/>
+      <tableStyleElement type="secondRowStripe" dxfId="5"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="比賽逐場費用明細-style 2">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="比賽逐場費用明細-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -640,58 +795,58 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D38" displayName="颶風騎士2026收支費用表格_3" name="颶風騎士2026收支費用表格_3" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="颶風騎士2026收支費用表格_3" displayName="颶風騎士2026收支費用表格_3" ref="A1:D38">
   <tableColumns count="4">
-    <tableColumn name="球員姓名" id="1"/>
-    <tableColumn name="隊費" id="2"/>
-    <tableColumn name="比賽儲值金" id="3"/>
-    <tableColumn name="狀態" id="4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="球員姓名"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="隊費"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="比賽儲值金"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="狀態"/>
   </tableColumns>
-  <tableStyleInfo name="隊費及儲值金收費紀錄-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="隊費及儲值金收費紀錄-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:L38" displayName="颶風騎士2026收支費用表格" name="颶風騎士2026收支費用表格" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="颶風騎士2026收支費用表格" displayName="颶風騎士2026收支費用表格" ref="A1:L38">
   <tableColumns count="12">
-    <tableColumn name="球員姓名" id="1"/>
-    <tableColumn name="比賽儲值金" id="2"/>
-    <tableColumn name="儲值金餘額" id="3"/>
-    <tableColumn name="比賽日3/8 （八里熱身賽）_x000a_(總費用: 1900)" id="4"/>
-    <tableColumn name="比賽日3/29 (瓊林熱身賽)_x000a_(總費用: 1920 )" id="5"/>
-    <tableColumn name="比賽日4/26 (VS TNT)_x000a_(總費用: 2943) _x000a_ " id="6"/>
-    <tableColumn name="比賽日5/3 (VS 卡吐司)_x000a_(總費用:  _x000a_ 2859)" id="7"/>
-    <tableColumn name="比賽日5/24 (VS 宙斯Z )_x000a_(總費用:  _x000a_ 2943)" id="8"/>
-    <tableColumn name="比賽日6/7 (VS 夢想家 )_x000a_(總費用:  _x000a_ 2943)" id="9"/>
-    <tableColumn name="比賽日7/19 (VS 紅閃電)_x000a_(總費用:  _x000a_ 3050）" id="10"/>
-    <tableColumn name="Column 12比賽日8/2 (VS 戰神)_x000a_(總費用:  _x000a_ 2946）" id="11"/>
-    <tableColumn name="比賽日8/30 (VS 戰神)_x000a_(總費用:  _x000a_ 2950）" id="12"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="球員姓名"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="比賽儲值金"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="儲值金餘額"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="比賽日3/8 （八里熱身賽）_x000a_(總費用: 1900)"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="比賽日3/29 (瓊林熱身賽)_x000a_(總費用: 1920 )"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="比賽日4/26 (VS TNT)_x000a_(總費用: 2943) _x000a_ "/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="比賽日5/3 (VS 卡吐司)_x000a_(總費用:  _x000a_ 2859)"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="比賽日5/24 (VS 宙斯Z )_x000a_(總費用:  _x000a_ 2943)"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="比賽日6/7 (VS 夢想家 )_x000a_(總費用:  _x000a_ 2943)"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="比賽日7/19 (VS 紅閃電)_x000a_(總費用:  _x000a_ 3050）"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Column 12比賽日8/2 (VS 戰神)_x000a_(總費用:  _x000a_ 2946）"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="比賽日8/30 (VS 戰神)_x000a_(總費用:  _x000a_ 2950）"/>
   </tableColumns>
-  <tableStyleInfo name="比賽逐場費用明細-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="比賽逐場費用明細-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="U1:U38" displayName="儲值金紀錄" name="儲值金紀錄" id="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="儲值金紀錄" displayName="儲值金紀錄" ref="U1:U38">
   <tableColumns count="1">
-    <tableColumn name="比賽儲值金_x000a_加值紀錄_x000a__x000a_(金額)" id="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="比賽儲值金_x000a_加值紀錄_x000a__x000a_(金額)"/>
   </tableColumns>
-  <tableStyleInfo name="比賽逐場費用明細-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="比賽逐場費用明細-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B34" displayName="颶風騎士2026收支費用表格_2" name="颶風騎士2026收支費用表格_2" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="颶風騎士2026收支費用表格_2" displayName="颶風騎士2026收支費用表格_2" ref="A1:B34">
   <tableColumns count="2">
-    <tableColumn name="日期 / 項目" id="1"/>
-    <tableColumn name="收入/支出金額" id="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="日期 / 項目"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="收入/支出金額"/>
   </tableColumns>
-  <tableStyleInfo name="隊費明細-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="隊費明細-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -881,23 +1036,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D38"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.25"/>
-    <col customWidth="1" min="2" max="2" width="7.0"/>
-    <col customWidth="1" min="3" max="3" width="9.13"/>
-    <col customWidth="1" min="4" max="4" width="15.13"/>
+    <col min="1" max="1" width="13.21875" customWidth="1"/>
+    <col min="2" max="2" width="7" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="69.75" customHeight="1">
+    <row r="1" spans="1:4" ht="69.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -911,548 +1069,550 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C2" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C3" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
+    <row r="4" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C4" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
+    <row r="5" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B5" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C5" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
+    <row r="6" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C6" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
+    <row r="7" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B7" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C7" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
+    <row r="8" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B8" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C8" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
+    <row r="9" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B9" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C9" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
+    <row r="10" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B10" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C10" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
+    <row r="11" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B11" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C11" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
+    <row r="12" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B12" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C12" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
+    <row r="13" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B13" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C13" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
+    <row r="14" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B14" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C14" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
+    <row r="15" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B15" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C15" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
+    <row r="16" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
         <v>34</v>
       </c>
       <c r="B16" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C16" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
+    <row r="17" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
         <v>35</v>
       </c>
       <c r="B17" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C17" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
+    <row r="18" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B18" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C18" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
+    <row r="19" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
         <v>37</v>
       </c>
       <c r="B19" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C19" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="20" ht="22.5" customHeight="1">
+    <row r="20" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
         <v>38</v>
       </c>
       <c r="B20" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C20" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" ht="22.5" customHeight="1">
+    <row r="21" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="25" t="s">
         <v>40</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="22" ht="22.5" customHeight="1">
+    <row r="22" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B22" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C22" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="23" ht="22.5" customHeight="1">
+    <row r="23" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
         <v>44</v>
       </c>
       <c r="B23" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C23" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="24" ht="22.5" customHeight="1">
+    <row r="24" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
         <v>45</v>
       </c>
       <c r="B24" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C24" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="25" ht="22.5" customHeight="1">
+    <row r="25" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>46</v>
       </c>
       <c r="B25" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C25" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" ht="22.5" customHeight="1">
+    <row r="26" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B26" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C26" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="27" ht="22.5" customHeight="1">
+    <row r="27" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="4" t="s">
         <v>48</v>
       </c>
       <c r="B27" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C27" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="28" ht="22.5" customHeight="1">
+    <row r="28" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
         <v>49</v>
       </c>
       <c r="B28" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C28" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D28" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29" ht="22.5" customHeight="1">
+    <row r="29" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
         <v>50</v>
       </c>
       <c r="B29" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C29" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="30" ht="22.5" customHeight="1">
+    <row r="30" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="31" ht="22.5" customHeight="1">
+    <row r="31" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
         <v>52</v>
       </c>
       <c r="B31" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C31" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="32" ht="22.5" customHeight="1">
+    <row r="32" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B32" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C32" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="33" ht="22.5" customHeight="1">
+    <row r="33" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B33" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C33" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="34" ht="22.5" customHeight="1">
+    <row r="34" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B34" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C34" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="35" ht="22.5" customHeight="1">
+    <row r="35" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="25" t="s">
         <v>56</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="5">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="36" ht="22.5" customHeight="1">
+    <row r="36" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="25" t="s">
         <v>57</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="5">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="37" ht="22.5" customHeight="1">
+    <row r="37" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="25" t="s">
         <v>58</v>
       </c>
       <c r="B37" s="5"/>
       <c r="C37" s="5">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="38" ht="22.5" customHeight="1">
+    <row r="38" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="4" t="s">
         <v>59</v>
       </c>
       <c r="B38" s="5">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="C38" s="5">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D38" s="7" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D38">
+  <phoneticPr fontId="5" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D38" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"已繳納,未繳納"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:A38"/>
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:A38" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:U38"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.25"/>
-    <col customWidth="1" min="2" max="2" width="9.13"/>
-    <col customWidth="1" min="3" max="3" width="11.0"/>
-    <col customWidth="1" min="4" max="4" width="25.63"/>
-    <col customWidth="1" min="5" max="5" width="20.5"/>
-    <col customWidth="1" min="6" max="6" width="21.63"/>
-    <col customWidth="1" min="7" max="7" width="22.25"/>
-    <col customWidth="1" min="8" max="8" width="22.88"/>
-    <col customWidth="1" min="9" max="12" width="24.13"/>
-    <col customWidth="1" min="21" max="21" width="18.63"/>
+    <col min="1" max="1" width="13.21875" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="25.609375" customWidth="1"/>
+    <col min="5" max="5" width="20.5" customWidth="1"/>
+    <col min="6" max="6" width="21.609375" customWidth="1"/>
+    <col min="7" max="7" width="22.21875" customWidth="1"/>
+    <col min="8" max="8" width="22.88671875" customWidth="1"/>
+    <col min="9" max="12" width="24.109375" customWidth="1"/>
+    <col min="21" max="21" width="18.609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="69.75" customHeight="1">
+    <row r="1" spans="1:21" ht="69.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1493,25 +1653,25 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="10" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C2" s="12">
-        <f t="shared" ref="C2:C38" si="1">B2-D2-E2-F2-G2-H2-I2-J2-K2-L2-M2-N2-O2-P2-Q2-R2-S2-T2+U2</f>
+        <f t="shared" ref="C2:C38" si="0">B2-D2-E2-F2-G2-H2-I2-J2-K2-L2-M2-N2-O2-P2-Q2-R2-S2-T2+U2</f>
         <v>1609</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
       <c r="H2" s="11">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="I2" s="13"/>
       <c r="J2" s="14"/>
@@ -1519,75 +1679,75 @@
       <c r="L2" s="15"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1059</v>
       </c>
       <c r="D3" s="12"/>
       <c r="E3" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F3" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G3" s="11"/>
       <c r="H3" s="11">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="I3" s="16"/>
       <c r="J3" s="17"/>
       <c r="K3" s="18">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L3" s="19"/>
       <c r="U3" s="5"/>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
+    <row r="4" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C4" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1126</v>
       </c>
       <c r="D4" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H4" s="11">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="I4" s="20"/>
       <c r="J4" s="21"/>
       <c r="K4" s="21"/>
       <c r="L4" s="22">
-        <v>312.0</v>
+        <v>312</v>
       </c>
       <c r="U4" s="5"/>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
+    <row r="5" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B5" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C5" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="D5" s="12"/>
@@ -1601,119 +1761,119 @@
       <c r="L5" s="27"/>
       <c r="U5" s="5"/>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
+    <row r="6" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="10" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C6" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>206</v>
       </c>
       <c r="D6" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E6" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F6" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G6" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H6" s="11">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="I6" s="29">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="J6" s="30"/>
       <c r="K6" s="30">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L6" s="31">
-        <v>312.0</v>
+        <v>312</v>
       </c>
       <c r="U6" s="5"/>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
+    <row r="7" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="10" t="s">
         <v>25</v>
       </c>
       <c r="B7" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C7" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>793</v>
       </c>
       <c r="D7" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E7" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
       <c r="I7" s="24"/>
       <c r="J7" s="18">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="K7" s="18">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L7" s="32">
-        <v>312.0</v>
+        <v>312</v>
       </c>
       <c r="U7" s="5"/>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
+    <row r="8" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="10" t="s">
         <v>26</v>
       </c>
       <c r="B8" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C8" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>453</v>
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F8" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G8" s="11">
-        <v>246.0</v>
+        <v>246</v>
       </c>
       <c r="H8" s="11"/>
       <c r="I8" s="20"/>
       <c r="J8" s="30">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="K8" s="30">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L8" s="31">
-        <v>312.0</v>
+        <v>312</v>
       </c>
       <c r="U8" s="5"/>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
+    <row r="9" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="10" t="s">
         <v>27</v>
       </c>
       <c r="B9" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C9" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="D9" s="12"/>
@@ -1727,47 +1887,47 @@
       <c r="L9" s="27"/>
       <c r="U9" s="5"/>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
+    <row r="10" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="10" t="s">
         <v>28</v>
       </c>
       <c r="B10" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C10" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>910</v>
       </c>
       <c r="D10" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E10" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F10" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G10" s="11">
-        <v>246.0</v>
+        <v>246</v>
       </c>
       <c r="H10" s="11"/>
       <c r="I10" s="20"/>
       <c r="J10" s="21"/>
       <c r="K10" s="21"/>
       <c r="L10" s="22">
-        <v>312.0</v>
+        <v>312</v>
       </c>
       <c r="U10" s="5"/>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
+    <row r="11" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="10" t="s">
         <v>29</v>
       </c>
       <c r="B11" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C11" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="D11" s="12"/>
@@ -1781,15 +1941,15 @@
       <c r="L11" s="27"/>
       <c r="U11" s="5"/>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
+    <row r="12" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="10" t="s">
         <v>30</v>
       </c>
       <c r="B12" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C12" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="D12" s="12"/>
@@ -1803,52 +1963,52 @@
       <c r="L12" s="33"/>
       <c r="U12" s="5"/>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
+    <row r="13" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B13" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C13" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>717</v>
       </c>
       <c r="D13" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E13" s="12"/>
       <c r="F13" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G13" s="11">
-        <v>246.0</v>
+        <v>246</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="34"/>
       <c r="J13" s="35">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="K13" s="35">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L13" s="19"/>
       <c r="U13" s="5"/>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
+    <row r="14" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="10" t="s">
         <v>32</v>
       </c>
       <c r="B14" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C14" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1886</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -1859,15 +2019,15 @@
       <c r="L14" s="33"/>
       <c r="U14" s="5"/>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
+    <row r="15" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="10" t="s">
         <v>33</v>
       </c>
       <c r="B15" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C15" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1861</v>
       </c>
       <c r="D15" s="12"/>
@@ -1875,7 +2035,7 @@
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
       <c r="H15" s="11">
-        <v>139.0</v>
+        <v>139</v>
       </c>
       <c r="I15" s="24"/>
       <c r="J15" s="26"/>
@@ -1883,51 +2043,51 @@
       <c r="L15" s="27"/>
       <c r="U15" s="5"/>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
+    <row r="16" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="10" t="s">
         <v>34</v>
       </c>
       <c r="B16" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C16" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>285</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
       <c r="F16" s="11">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="G16" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H16" s="11">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="I16" s="29">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="J16" s="30">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="K16" s="30">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L16" s="31">
-        <v>312.0</v>
+        <v>312</v>
       </c>
       <c r="U16" s="5"/>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
+    <row r="17" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="10" t="s">
         <v>35</v>
       </c>
       <c r="B17" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C17" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1706</v>
       </c>
       <c r="D17" s="12"/>
@@ -1938,30 +2098,30 @@
       <c r="I17" s="24"/>
       <c r="J17" s="26"/>
       <c r="K17" s="18">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L17" s="19"/>
       <c r="U17" s="5"/>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
+    <row r="18" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="10" t="s">
         <v>36</v>
       </c>
       <c r="B18" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C18" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1467</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
       <c r="F18" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G18" s="11"/>
       <c r="H18" s="11">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="I18" s="36"/>
       <c r="J18" s="37"/>
@@ -1969,139 +2129,139 @@
       <c r="L18" s="38"/>
       <c r="U18" s="5"/>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
+    <row r="19" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="10" t="s">
         <v>37</v>
       </c>
       <c r="B19" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C19" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1368</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F19" s="12"/>
       <c r="G19" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H19" s="11">
-        <v>139.0</v>
+        <v>139</v>
       </c>
       <c r="I19" s="39">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="J19" s="35"/>
       <c r="K19" s="35"/>
       <c r="L19" s="40"/>
       <c r="U19" s="5"/>
     </row>
-    <row r="20" ht="22.5" customHeight="1">
+    <row r="20" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="B20" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C20" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1267</v>
       </c>
       <c r="D20" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E20" s="12"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
       <c r="H20" s="11">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="I20" s="13"/>
       <c r="J20" s="14"/>
       <c r="K20" s="41">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L20" s="42"/>
       <c r="U20" s="5"/>
     </row>
-    <row r="21" ht="22.5" customHeight="1">
+    <row r="21" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="10" t="s">
         <v>43</v>
       </c>
       <c r="B21" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C21" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1020</v>
       </c>
       <c r="D21" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E21" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F21" s="11">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="G21" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H21" s="11"/>
       <c r="I21" s="39">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="J21" s="35">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="K21" s="35"/>
       <c r="L21" s="40"/>
       <c r="U21" s="5"/>
     </row>
-    <row r="22" ht="22.5" customHeight="1">
+    <row r="22" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="10" t="s">
         <v>44</v>
       </c>
       <c r="B22" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C22" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>728</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="12"/>
       <c r="F22" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G22" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H22" s="11"/>
       <c r="I22" s="29">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="J22" s="30">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="K22" s="30"/>
       <c r="L22" s="22">
-        <v>312.0</v>
+        <v>312</v>
       </c>
       <c r="U22" s="5"/>
     </row>
-    <row r="23" ht="22.5" customHeight="1">
+    <row r="23" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B23" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C23" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="D23" s="12"/>
@@ -2115,21 +2275,21 @@
       <c r="L23" s="27"/>
       <c r="U23" s="5"/>
     </row>
-    <row r="24" ht="22.5" customHeight="1">
+    <row r="24" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="10" t="s">
         <v>46</v>
       </c>
       <c r="B24" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C24" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1872</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="12"/>
       <c r="F24" s="11">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="G24" s="11"/>
       <c r="H24" s="11"/>
@@ -2139,86 +2299,86 @@
       <c r="L24" s="38"/>
       <c r="U24" s="5"/>
     </row>
-    <row r="25" ht="22.5" customHeight="1">
+    <row r="25" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="10" t="s">
         <v>47</v>
       </c>
       <c r="B25" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C25" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1317</v>
       </c>
       <c r="D25" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E25" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F25" s="11">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="G25" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H25" s="11"/>
       <c r="I25" s="34"/>
       <c r="J25" s="43"/>
       <c r="K25" s="43"/>
       <c r="L25" s="44">
-        <v>156.0</v>
+        <v>156</v>
       </c>
       <c r="U25" s="5"/>
     </row>
-    <row r="26" ht="22.5" customHeight="1">
+    <row r="26" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="10" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C26" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>931</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F26" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G26" s="11">
-        <v>246.0</v>
+        <v>246</v>
       </c>
       <c r="H26" s="11"/>
       <c r="I26" s="29">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="J26" s="30">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="K26" s="30"/>
       <c r="L26" s="38"/>
       <c r="U26" s="5"/>
     </row>
-    <row r="27" ht="22.5" customHeight="1">
+    <row r="27" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B27" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C27" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1754</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="12"/>
       <c r="F27" s="12"/>
       <c r="G27" s="11">
-        <v>246.0</v>
+        <v>246</v>
       </c>
       <c r="H27" s="11"/>
       <c r="I27" s="20"/>
@@ -2227,15 +2387,15 @@
       <c r="L27" s="38"/>
       <c r="U27" s="5"/>
     </row>
-    <row r="28" ht="22.5" customHeight="1">
+    <row r="28" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="10" t="s">
         <v>53</v>
       </c>
       <c r="B28" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C28" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="D28" s="12"/>
@@ -2249,54 +2409,54 @@
       <c r="L28" s="27"/>
       <c r="U28" s="5"/>
     </row>
-    <row r="29" ht="22.5" customHeight="1">
+    <row r="29" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="10" t="s">
         <v>54</v>
       </c>
       <c r="B29" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C29" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1094</v>
       </c>
       <c r="D29" s="11">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="E29" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F29" s="11">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="G29" s="11">
-        <v>246.0</v>
+        <v>246</v>
       </c>
       <c r="H29" s="11"/>
       <c r="I29" s="29">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="J29" s="30"/>
       <c r="K29" s="30"/>
       <c r="L29" s="38"/>
       <c r="U29" s="5"/>
     </row>
-    <row r="30" ht="22.5" customHeight="1">
+    <row r="30" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="10" t="s">
         <v>55</v>
       </c>
       <c r="B30" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C30" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1877</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="12"/>
       <c r="F30" s="12"/>
       <c r="G30" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H30" s="11"/>
       <c r="I30" s="34"/>
@@ -2305,24 +2465,24 @@
       <c r="L30" s="40"/>
       <c r="U30" s="5"/>
     </row>
-    <row r="31" ht="22.5" customHeight="1">
+    <row r="31" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="10" t="s">
         <v>49</v>
       </c>
       <c r="B31" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C31" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1763</v>
       </c>
       <c r="D31" s="12"/>
       <c r="E31" s="11">
-        <v>114.0</v>
+        <v>114</v>
       </c>
       <c r="F31" s="12"/>
       <c r="G31" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H31" s="11"/>
       <c r="I31" s="20"/>
@@ -2331,49 +2491,49 @@
       <c r="L31" s="38"/>
       <c r="U31" s="5"/>
     </row>
-    <row r="32" ht="22.5" customHeight="1">
+    <row r="32" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="10" t="s">
         <v>50</v>
       </c>
       <c r="B32" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C32" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>541</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="11"/>
       <c r="F32" s="11">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="G32" s="11">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="H32" s="11">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="I32" s="34"/>
       <c r="J32" s="35">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="K32" s="35">
-        <v>294.0</v>
+        <v>294</v>
       </c>
       <c r="L32" s="32">
-        <v>312.0</v>
+        <v>312</v>
       </c>
       <c r="U32" s="5"/>
     </row>
-    <row r="33" ht="22.5" customHeight="1">
+    <row r="33" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="10" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="C33" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="D33" s="12"/>
@@ -2387,22 +2547,22 @@
       <c r="L33" s="33"/>
       <c r="U33" s="5"/>
     </row>
-    <row r="34" ht="22.5" customHeight="1">
+    <row r="34" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="45" t="s">
         <v>56</v>
       </c>
       <c r="B34" s="11">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="C34" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>900</v>
       </c>
       <c r="D34" s="11">
-        <v>300.0</v>
+        <v>300</v>
       </c>
       <c r="E34" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
@@ -2410,54 +2570,54 @@
       <c r="I34" s="24"/>
       <c r="J34" s="26"/>
       <c r="K34" s="18">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="L34" s="19"/>
       <c r="U34" s="5"/>
     </row>
-    <row r="35" ht="22.5" customHeight="1">
+    <row r="35" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="45" t="s">
         <v>40</v>
       </c>
       <c r="B35" s="11">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="C35" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>600</v>
       </c>
       <c r="D35" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="E35" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
       <c r="H35" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="I35" s="13"/>
       <c r="J35" s="41">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="K35" s="41">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="L35" s="31">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="U35" s="5"/>
     </row>
-    <row r="36" ht="22.5" customHeight="1">
+    <row r="36" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="45" t="s">
         <v>57</v>
       </c>
       <c r="B36" s="11">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="C36" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1200</v>
       </c>
       <c r="D36" s="11"/>
@@ -2465,100 +2625,102 @@
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
       <c r="H36" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="I36" s="41">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="J36" s="41"/>
       <c r="K36" s="41"/>
       <c r="L36" s="40"/>
       <c r="U36" s="5"/>
     </row>
-    <row r="37" ht="22.5" customHeight="1">
+    <row r="37" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="45" t="s">
         <v>58</v>
       </c>
       <c r="B37" s="11">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="C37" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>900</v>
       </c>
       <c r="D37" s="11"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="H37" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="I37" s="34"/>
       <c r="J37" s="35">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="K37" s="35"/>
       <c r="L37" s="22">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="U37" s="5"/>
     </row>
-    <row r="38" ht="22.5" customHeight="1">
+    <row r="38" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="45" t="s">
         <v>51</v>
       </c>
       <c r="B38" s="11">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="C38" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>900</v>
       </c>
       <c r="D38" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="E38" s="11">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="F38" s="12"/>
       <c r="G38" s="12"/>
       <c r="H38" s="11"/>
       <c r="I38" s="46">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="J38" s="41">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="K38" s="41"/>
       <c r="L38" s="47"/>
       <c r="U38" s="5"/>
     </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:A38"/>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:A38" xr:uid="{00000000-0002-0000-0100-000000000000}"/>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId4"/>
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D34"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="24.13"/>
-    <col customWidth="1" min="2" max="2" width="17.75"/>
+    <col min="1" max="1" width="24.109375" customWidth="1"/>
+    <col min="2" max="2" width="17.71875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2569,165 +2731,166 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="5">
-        <v>400.0</v>
+        <v>400</v>
       </c>
       <c r="D2" s="23">
         <f>-SUM(颶風騎士2026收支費用表格_2[收入/支出金額])</f>
         <v>-1936</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>39</v>
       </c>
       <c r="B3" s="5">
-        <v>310.0</v>
-      </c>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>41</v>
       </c>
       <c r="B4" s="5">
-        <v>710.0</v>
-      </c>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B5" s="5">
-        <v>516.0</v>
-      </c>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="4"/>
       <c r="B6" s="28"/>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
+    <row r="7" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="4"/>
       <c r="B7" s="28"/>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
+    <row r="8" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="4"/>
       <c r="B8" s="28"/>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
+    <row r="9" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4"/>
       <c r="B9" s="28"/>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
+    <row r="10" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="4"/>
       <c r="B10" s="28"/>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
+    <row r="11" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="4"/>
       <c r="B11" s="28"/>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
+    <row r="12" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4"/>
       <c r="B12" s="28"/>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
+    <row r="13" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4"/>
       <c r="B13" s="28"/>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
+    <row r="14" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4"/>
       <c r="B14" s="28"/>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
+    <row r="15" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="4"/>
       <c r="B15" s="28"/>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
+    <row r="16" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="4"/>
       <c r="B16" s="28"/>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
+    <row r="17" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="4"/>
       <c r="B17" s="28"/>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
+    <row r="18" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="4"/>
       <c r="B18" s="28"/>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
+    <row r="19" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="4"/>
       <c r="B19" s="28"/>
     </row>
-    <row r="20" ht="22.5" customHeight="1">
+    <row r="20" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="4"/>
       <c r="B20" s="28"/>
     </row>
-    <row r="21" ht="22.5" customHeight="1">
+    <row r="21" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="4"/>
       <c r="B21" s="28"/>
     </row>
-    <row r="22" ht="22.5" customHeight="1">
+    <row r="22" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="4"/>
       <c r="B22" s="28"/>
     </row>
-    <row r="23" ht="22.5" customHeight="1">
+    <row r="23" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="4"/>
       <c r="B23" s="28"/>
     </row>
-    <row r="24" ht="22.5" customHeight="1">
+    <row r="24" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="4"/>
       <c r="B24" s="28"/>
     </row>
-    <row r="25" ht="22.5" customHeight="1">
+    <row r="25" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="4"/>
       <c r="B25" s="28"/>
     </row>
-    <row r="26" ht="22.5" customHeight="1">
+    <row r="26" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4"/>
       <c r="B26" s="28"/>
     </row>
-    <row r="27" ht="22.5" customHeight="1">
+    <row r="27" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="4"/>
       <c r="B27" s="28"/>
     </row>
-    <row r="28" ht="22.5" customHeight="1">
+    <row r="28" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4"/>
       <c r="B28" s="28"/>
     </row>
-    <row r="29" ht="22.5" customHeight="1">
+    <row r="29" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4"/>
       <c r="B29" s="28"/>
     </row>
-    <row r="30" ht="22.5" customHeight="1">
+    <row r="30" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="4"/>
       <c r="B30" s="28"/>
     </row>
-    <row r="31" ht="22.5" customHeight="1">
+    <row r="31" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="4"/>
       <c r="B31" s="28"/>
     </row>
-    <row r="32" ht="22.5" customHeight="1">
+    <row r="32" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4"/>
       <c r="B32" s="28"/>
     </row>
-    <row r="33" ht="22.5" customHeight="1">
+    <row r="33" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="4"/>
       <c r="B33" s="28"/>
     </row>
-    <row r="34" ht="22.5" customHeight="1">
+    <row r="34" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="4"/>
       <c r="B34" s="28"/>
     </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:A34"/>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:A34" xr:uid="{00000000-0002-0000-0200-000000000000}"/>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>